<commit_message>
refactor: 엑셀 폼 수정
</commit_message>
<xml_diff>
--- a/src/main/resources/sheet/column-decision.xlsx
+++ b/src/main/resources/sheet/column-decision.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/junbeom/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/junbeom/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F21CB60-9550-114A-A1F5-A60622EC9C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A384A3E5-6968-3A4A-94C4-0CF33117DE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,15 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
   <si>
     <t>테이블명</t>
   </si>
   <si>
     <t>컬럼명</t>
-  </si>
-  <si>
-    <t>마스킹</t>
   </si>
   <si>
     <t>방식</t>
@@ -240,7 +237,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -250,13 +247,13 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -593,14 +590,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:Q31"/>
+  <dimension ref="B2:P31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="9" width="18" customWidth="1"/>
+    <col min="2" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" ht="20">
+    <row r="2" spans="2:16" ht="20">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -622,20 +619,17 @@
       <c r="H2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="J2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-    </row>
-    <row r="3" spans="2:17" ht="17" customHeight="1">
+    </row>
+    <row r="3" spans="2:16" ht="17" customHeight="1">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -643,18 +637,17 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="K3" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="J3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" s="7"/>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-    </row>
-    <row r="4" spans="2:17">
+    </row>
+    <row r="4" spans="2:16">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -662,16 +655,15 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="K4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="7"/>
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-    </row>
-    <row r="5" spans="2:17">
+    </row>
+    <row r="5" spans="2:16">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -679,16 +671,15 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="K5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="7"/>
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
-    </row>
-    <row r="6" spans="2:17">
+    </row>
+    <row r="6" spans="2:16">
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -696,16 +687,15 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="K6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="7"/>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
-    </row>
-    <row r="7" spans="2:17">
+    </row>
+    <row r="7" spans="2:16">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -713,16 +703,15 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="K7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="7"/>
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
-      <c r="Q7" s="7"/>
-    </row>
-    <row r="8" spans="2:17">
+    </row>
+    <row r="8" spans="2:16">
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -730,16 +719,15 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="K8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="7"/>
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-    </row>
-    <row r="9" spans="2:17">
+    </row>
+    <row r="9" spans="2:16">
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -747,16 +735,15 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="K9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="7"/>
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
-    </row>
-    <row r="10" spans="2:17">
+    </row>
+    <row r="10" spans="2:16">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -764,16 +751,15 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="K10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="7"/>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-    </row>
-    <row r="11" spans="2:17">
+    </row>
+    <row r="11" spans="2:16">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -781,16 +767,15 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="K11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="7"/>
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
-    </row>
-    <row r="12" spans="2:17">
+    </row>
+    <row r="12" spans="2:16">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -798,16 +783,15 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="K12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="7"/>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-    </row>
-    <row r="13" spans="2:17">
+    </row>
+    <row r="13" spans="2:16">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -815,16 +799,15 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="K13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="7"/>
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-    </row>
-    <row r="14" spans="2:17">
+    </row>
+    <row r="14" spans="2:16">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -832,16 +815,15 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="K14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="7"/>
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-    </row>
-    <row r="15" spans="2:17">
+    </row>
+    <row r="15" spans="2:16">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -849,16 +831,15 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="K15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="7"/>
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-    </row>
-    <row r="16" spans="2:17">
+    </row>
+    <row r="16" spans="2:16">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -866,16 +847,15 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="K16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="7"/>
       <c r="L16" s="7"/>
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-    </row>
-    <row r="17" spans="2:17">
+    </row>
+    <row r="17" spans="2:16">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -883,16 +863,15 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="K17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="7"/>
       <c r="L17" s="7"/>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-    </row>
-    <row r="18" spans="2:17">
+    </row>
+    <row r="18" spans="2:16">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -900,9 +879,8 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="2:17">
+    </row>
+    <row r="19" spans="2:16">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -910,9 +888,8 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="2:17">
+    </row>
+    <row r="20" spans="2:16">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -920,9 +897,8 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="2:17">
+    </row>
+    <row r="21" spans="2:16">
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -930,9 +906,8 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="2:17">
+    </row>
+    <row r="22" spans="2:16">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -940,9 +915,8 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="2:17">
+    </row>
+    <row r="23" spans="2:16">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -950,9 +924,8 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="2:17">
+    </row>
+    <row r="24" spans="2:16">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -960,9 +933,8 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-    </row>
-    <row r="25" spans="2:17">
+    </row>
+    <row r="25" spans="2:16">
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -970,9 +942,8 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-    </row>
-    <row r="26" spans="2:17">
+    </row>
+    <row r="26" spans="2:16">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -980,9 +951,8 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="2:17">
+    </row>
+    <row r="27" spans="2:16">
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -990,9 +960,8 @@
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-    </row>
-    <row r="28" spans="2:17">
+    </row>
+    <row r="28" spans="2:16">
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -1000,9 +969,8 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="2:17">
+    </row>
+    <row r="29" spans="2:16">
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1010,9 +978,8 @@
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-    </row>
-    <row r="30" spans="2:17">
+    </row>
+    <row r="30" spans="2:16">
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -1020,9 +987,8 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-    </row>
-    <row r="31" spans="2:17">
+    </row>
+    <row r="31" spans="2:16">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1030,22 +996,18 @@
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="K2:Q2"/>
-    <mergeCell ref="K3:Q17"/>
+    <mergeCell ref="J2:P2"/>
+    <mergeCell ref="J3:P17"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D1002" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"Y,N"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E1002" xr:uid="{00000000-0002-0000-0000-000001000000}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D1002" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"부분 마스킹,해시,고정값"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F3:F1002" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E1002" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"앞에서부터,뒤에서부터"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1067,206 +1029,206 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
         <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>24</v>
       </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>26</v>
-      </c>
-      <c r="E6" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>